<commit_message>
feat(support): support international partner locations and geocoding workflow
</commit_message>
<xml_diff>
--- a/public/templates/rede-autorizada-nacional.xlsx
+++ b/public/templates/rede-autorizada-nacional.xlsx
@@ -415,12 +415,12 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Campos obrigatórios: Nome Fantasia, Fone, Cidade, UF, CEP, Endereço e Número.</v>
+        <v>Campos obrigatórios: Nome Fantasia, Cidade, País, Endereço e Número. Estado/Província e Código postal dependem do país.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>CEP: use 00000-000 ou 00000000.</v>
+        <v>País: use um dos códigos BR, US, AR, BO, CL, CO, EC, MX, PA, PY, PE, PR, DO, TT ou VE.</v>
       </c>
     </row>
     <row r="5">
@@ -440,12 +440,12 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Latitude e Longitude são opcionais e devem ser preenchidas juntas.</v>
+        <v>Latitude e Longitude não fazem parte do formato oficial.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Quando as coordenadas estiverem vazias, a API usará o centroide da cidade. A localização será aproximada.</v>
+        <v>Endereços importados serão geocodificados automaticamente; correções manuais são feitas no cadastro administrativo.</v>
       </c>
     </row>
     <row r="10">
@@ -462,7 +462,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:L1"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -475,8 +475,6 @@
     <col min="9" max="9" width="22.83203125" customWidth="1"/>
     <col min="10" max="10" width="22.83203125" customWidth="1"/>
     <col min="11" max="11" width="22.83203125" customWidth="1"/>
-    <col min="12" max="12" width="22.83203125" customWidth="1"/>
-    <col min="13" max="13" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -490,39 +488,36 @@
         <v>Cidade</v>
       </c>
       <c r="D1" t="str">
-        <v>UF</v>
+        <v>Estado/Província</v>
       </c>
       <c r="E1" t="str">
-        <v>CEP</v>
+        <v>País</v>
       </c>
       <c r="F1" t="str">
+        <v>Código postal</v>
+      </c>
+      <c r="G1" t="str">
         <v>Endereço</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Número</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>E-mail</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Site</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>Região</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Especialidade</v>
-      </c>
-      <c r="L1" t="str">
-        <v>Latitude</v>
-      </c>
-      <c r="M1" t="str">
-        <v>Longitude</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>